<commit_message>
Adding config documentation update and change excel file name
</commit_message>
<xml_diff>
--- a/Clases.xlsx
+++ b/Clases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maurobenetti/Documents/PhD/Python/ISEC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D850494-11E7-1244-BBF9-C04A61ACEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5846469-B0B3-7248-AC16-93CF416433B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16980" xr2:uid="{33521C79-F8DF-B042-8F80-16E98765405A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Name</t>
   </si>
@@ -44,13 +44,16 @@
     <t>Frequency</t>
   </si>
   <si>
-    <t>Limpia tapicería en espuma Binner</t>
-  </si>
-  <si>
-    <t>Limpia tapicería y alfombras Binner</t>
-  </si>
-  <si>
-    <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
+    <t>Limpiador Dr. Beckmann de alfombras 2 en 1 poder oxi x 650 ml</t>
+  </si>
+  <si>
+    <t>Limpiador de alfombras 2 en 1 Dr. Beckmann poder oxi x 650 ml</t>
+  </si>
+  <si>
+    <t>Limpiador Dr. Beckmann de tapiz 2 en 1 poder oxi x 650 ml</t>
+  </si>
+  <si>
+    <t>Ford Ranger XL 2.0L Diesel Cabina Doble 4x2 plan ovalo cuotas</t>
   </si>
 </sst>
 </file>
@@ -470,7 +473,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -478,7 +481,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>1</v>

</xml_diff>

<commit_message>
Enhance README and code to clarify penalized distance calculation; update cost matrices and add configuration files for semantic distance analysis.
</commit_message>
<xml_diff>
--- a/Clases.xlsx
+++ b/Clases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maurobenetti/Documents/PhD/Python/ISEC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5846469-B0B3-7248-AC16-93CF416433B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC67066-4516-4442-83A6-F4CD964C5E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16980" xr2:uid="{33521C79-F8DF-B042-8F80-16E98765405A}"/>
   </bookViews>
@@ -44,16 +44,16 @@
     <t>Frequency</t>
   </si>
   <si>
-    <t>Limpiador Dr. Beckmann de alfombras 2 en 1 poder oxi x 650 ml</t>
-  </si>
-  <si>
-    <t>Limpiador de alfombras 2 en 1 Dr. Beckmann poder oxi x 650 ml</t>
-  </si>
-  <si>
-    <t>Limpiador Dr. Beckmann de tapiz 2 en 1 poder oxi x 650 ml</t>
-  </si>
-  <si>
-    <t>Ford Ranger XL 2.0L Diesel Cabina Doble 4x2 plan ovalo cuotas</t>
+    <t>XDKT11T3</t>
+  </si>
+  <si>
+    <t>XDKG11T3</t>
+  </si>
+  <si>
+    <t>LDKT11T3</t>
+  </si>
+  <si>
+    <t>LDKT11T3QET</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: Introduce comprehensive parameter analysis, new application components, extensive testing, and detailed reporting with visualizations.
</commit_message>
<xml_diff>
--- a/Clases.xlsx
+++ b/Clases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maurobenetti/Documents/PhD/Python/ISEC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC67066-4516-4442-83A6-F4CD964C5E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BBA3C3-50A3-E943-B497-FFC1AA597A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16980" xr2:uid="{33521C79-F8DF-B042-8F80-16E98765405A}"/>
   </bookViews>
@@ -460,7 +460,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -468,7 +468,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -476,7 +476,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>